<commit_message>
Actualización del dashboard, scripts de análisis y nuevos archivos HTML
</commit_message>
<xml_diff>
--- a/Resultados_Analisis.xlsx
+++ b/Resultados_Analisis.xlsx
@@ -3174,7 +3174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3200,22 +3200,87 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Intercepto (Base)</t>
+          <t>Intercepto (Lunes)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Coef_Dia (J/V)</t>
+          <t>Coef_ADR</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Coef_ADR</t>
+          <t>P_Value_ADR</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>Coef_Partidas</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>P_Value_Partidas</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Coef_Dia_Martes</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>P_Value_Dia_Martes</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Coef_Dia_Miércoles</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>P_Value_Dia_Miércoles</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Coef_Dia_Jueves</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>P_Value_Dia_Jueves</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Coef_Dia_Viernes</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>P_Value_Dia_Viernes</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Coef_Dia_Sábado</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>P_Value_Dia_Sábado</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Coef_Dia_Domingo</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>P_Value_Dia_Domingo</t>
         </is>
       </c>
     </row>
@@ -3231,23 +3296,60 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.1260841813412206</v>
+        <v>0.1700756048173657</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3550833442182561</v>
+        <v>0.4124022366784226</v>
       </c>
       <c r="E2" t="n">
-        <v>60.53176555494666</v>
+        <v>47.68056979597748</v>
       </c>
       <c r="F2" t="n">
-        <v>39.04076958805842</v>
+        <v>-45.15536329301372</v>
       </c>
       <c r="G2" t="n">
-        <v>-48.78043701435605</v>
+        <v>9.786984442573144e-08</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.005812978440149</v>
-      </c>
+        <v>-1.659555771640722</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.3168579083446923</v>
+      </c>
+      <c r="J2" t="n">
+        <v>26.29253510043803</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.0003457435682699729</v>
+      </c>
+      <c r="L2" t="n">
+        <v>5.900805950266649</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.4107771442537137</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50.4361542655416</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1.211307418665193e-12</v>
+      </c>
+      <c r="P2" t="n">
+        <v>58.13616786297615</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1.579730722932461e-16</v>
+      </c>
+      <c r="R2" t="n">
+        <v>-13.90455585055715</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.300188642715837</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3261,22 +3363,61 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.09259960592953009</v>
+        <v>0.193307628544352</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3043018335954125</v>
+        <v>0.4396676341787646</v>
       </c>
       <c r="E3" t="n">
-        <v>1074.604663365436</v>
+        <v>1236.097578485026</v>
       </c>
       <c r="F3" t="n">
-        <v>-469.7192712494751</v>
+        <v>185.4785538817347</v>
       </c>
       <c r="G3" t="n">
-        <v>282.4470180035889</v>
+        <v>0.1604063712592375</v>
       </c>
       <c r="H3" t="n">
-        <v>-3.95839181641032</v>
+        <v>-13.5573787638421</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.4569269525828857</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-321.6279870919607</v>
+      </c>
+      <c r="K3" t="n">
+        <v>3.50702365706393e-06</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-91.00230357657213</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.1783760790666857</v>
+      </c>
+      <c r="N3" t="n">
+        <v>-424.2322581810427</v>
+      </c>
+      <c r="O3" t="n">
+        <v>3.882849554315895e-10</v>
+      </c>
+      <c r="P3" t="n">
+        <v>-1048.836170670652</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1.619440786411632e-38</v>
+      </c>
+      <c r="R3" t="n">
+        <v>266.7310295885878</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.1153051335489899</v>
+      </c>
+      <c r="T3" t="n">
+        <v>-1080.310684665819</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.1175967627415802</v>
       </c>
     </row>
     <row r="4">
@@ -3291,21 +3432,56 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.03389866380547268</v>
+        <v>0.05560914704296582</v>
       </c>
       <c r="D4" t="n">
-        <v>0.184115897753216</v>
+        <v>0.2358159177048187</v>
       </c>
       <c r="E4" t="n">
-        <v>147.2733538940021</v>
+        <v>120.5923941977287</v>
       </c>
       <c r="F4" t="n">
-        <v>23.29774624731415</v>
+        <v>96.07329096170477</v>
       </c>
       <c r="G4" t="n">
-        <v>98.41987824549875</v>
+        <v>8.705686020247343e-09</v>
       </c>
       <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>24.48205825355889</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.01261046200109553</v>
+      </c>
+      <c r="L4" t="n">
+        <v>43.89880876929961</v>
+      </c>
+      <c r="M4" t="n">
+        <v>9.031578284966896e-06</v>
+      </c>
+      <c r="N4" t="n">
+        <v>61.18858116120788</v>
+      </c>
+      <c r="O4" t="n">
+        <v>9.618124971307175e-11</v>
+      </c>
+      <c r="P4" t="n">
+        <v>36.35484296597966</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.0001213232519168389</v>
+      </c>
+      <c r="R4" t="n">
+        <v>94.8774325937605</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.0001096822567259881</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3319,23 +3495,58 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.03002070225083076</v>
+        <v>0.03205848715389004</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1732648327007842</v>
+        <v>0.179048840135562</v>
       </c>
       <c r="E5" t="n">
-        <v>37.39810033336489</v>
+        <v>36.60821475481659</v>
       </c>
       <c r="F5" t="n">
-        <v>6.476882508725272</v>
+        <v>-0.09313140934386192</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.100678021951173</v>
+        <v>0.9320836406602899</v>
       </c>
       <c r="H5" t="n">
-        <v>3.197733868083656</v>
-      </c>
+        <v>3.213164568735684</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5.154715080915779e-38</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3.10494428631974</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.007023759106298298</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-1.029686364858212</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.3730751393339292</v>
+      </c>
+      <c r="N5" t="n">
+        <v>7.573679940830623</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1.700261728840028e-10</v>
+      </c>
+      <c r="P5" t="n">
+        <v>6.870522319464734</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1.332834684538849e-08</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3349,23 +3560,58 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.07795077189013466</v>
+        <v>0.1089837606996321</v>
       </c>
       <c r="D6" t="n">
-        <v>0.279196654511</v>
+        <v>0.3301268857570254</v>
       </c>
       <c r="E6" t="n">
-        <v>451.327184676828</v>
+        <v>421.5441744285457</v>
       </c>
       <c r="F6" t="n">
-        <v>-165.6290803116082</v>
+        <v>628.1796234179218</v>
       </c>
       <c r="G6" t="n">
-        <v>633.2230887991782</v>
+        <v>4.918120427504847e-75</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.8298366203051644</v>
-      </c>
+        <v>-0.9344348406480867</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.8272800372236214</v>
+      </c>
+      <c r="J6" t="n">
+        <v>36.44647891439327</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.08248261305533817</v>
+      </c>
+      <c r="L6" t="n">
+        <v>50.44459516209241</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.01628330905860271</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-0.4731120939261686</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.9820593951516643</v>
+      </c>
+      <c r="P6" t="n">
+        <v>-300.1852449595614</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>2.266639926006222e-41</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3379,21 +3625,54 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.01789237617649864</v>
+        <v>0.02057542591281936</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1337623870020965</v>
+        <v>0.1434413675088862</v>
       </c>
       <c r="E7" t="n">
-        <v>103.9592581286586</v>
+        <v>100.5847592916408</v>
       </c>
       <c r="F7" t="n">
-        <v>13.95173960884621</v>
+        <v>48.14003295876176</v>
       </c>
       <c r="G7" t="n">
-        <v>48.32019463044599</v>
+        <v>1.100311630455323e-24</v>
       </c>
       <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>11.38088177722525</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.000347559828579288</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-2.156931322152675</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.5041525076748478</v>
+      </c>
+      <c r="N7" t="n">
+        <v>16.0887188606706</v>
+      </c>
+      <c r="O7" t="n">
+        <v>4.631654321640435e-07</v>
+      </c>
+      <c r="P7" t="n">
+        <v>18.6652273261719</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>8.595039467518627e-09</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3407,23 +3686,58 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.008220153826506427</v>
+        <v>0.009316055991454131</v>
       </c>
       <c r="D8" t="n">
-        <v>0.09066506398004927</v>
+        <v>0.09651971814843914</v>
       </c>
       <c r="E8" t="n">
-        <v>30.41395645258213</v>
+        <v>30.10536100726337</v>
       </c>
       <c r="F8" t="n">
-        <v>1.769302486996937</v>
+        <v>-3.782644297483694</v>
       </c>
       <c r="G8" t="n">
-        <v>-3.811919375256882</v>
+        <v>1.359144789920089e-10</v>
       </c>
       <c r="H8" t="n">
-        <v>1.043393640273994</v>
-      </c>
+        <v>1.044528820520656</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3.185817852874984e-17</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.4746349739028046</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.4441820354350638</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1.78952374669203</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.003546285612992183</v>
+      </c>
+      <c r="N8" t="n">
+        <v>3.169152084533057</v>
+      </c>
+      <c r="O8" t="n">
+        <v>2.902084651450133e-07</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.9646363363987482</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.1198785445627527</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3437,23 +3751,58 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.1072543352147737</v>
+        <v>0.1239535878572392</v>
       </c>
       <c r="D9" t="n">
-        <v>0.3274970766507293</v>
+        <v>0.3520704302511632</v>
       </c>
       <c r="E9" t="n">
-        <v>592.6999184888249</v>
+        <v>561.7671640173904</v>
       </c>
       <c r="F9" t="n">
-        <v>-247.7051177123309</v>
+        <v>659.3375904143591</v>
       </c>
       <c r="G9" t="n">
-        <v>675.1154950120442</v>
+        <v>7.162837399924625e-171</v>
       </c>
       <c r="H9" t="n">
-        <v>-11.28706877449386</v>
-      </c>
+        <v>-11.46374780634596</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.01407881215068237</v>
+      </c>
+      <c r="J9" t="n">
+        <v>62.93025879941565</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.008549450142134343</v>
+      </c>
+      <c r="L9" t="n">
+        <v>188.892902853048</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2.386943745701964e-15</v>
+      </c>
+      <c r="N9" t="n">
+        <v>-67.82663537550943</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.003873682069631895</v>
+      </c>
+      <c r="P9" t="n">
+        <v>-401.776376223977</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>3.774859572878946e-53</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3467,21 +3816,54 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.0002303473893709995</v>
+        <v>0.009758013470693494</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01517719965510764</v>
+        <v>0.09878265774260933</v>
       </c>
       <c r="E10" t="n">
-        <v>120.5669732882632</v>
+        <v>118.6625549724603</v>
       </c>
       <c r="F10" t="n">
-        <v>-1.838086909137385</v>
+        <v>-2.980526805680263</v>
       </c>
       <c r="G10" t="n">
-        <v>-3.609858007689155</v>
+        <v>0.2382838538210327</v>
       </c>
       <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>6.981559707167488</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.002169941670626501</v>
+      </c>
+      <c r="L10" t="n">
+        <v>7.153455500135223</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.001900541367305897</v>
+      </c>
+      <c r="N10" t="n">
+        <v>16.23644488838811</v>
+      </c>
+      <c r="O10" t="n">
+        <v>6.523896473640382e-13</v>
+      </c>
+      <c r="P10" t="n">
+        <v>-15.83487968221744</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1.45975345198215e-12</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3501,17 +3883,44 @@
         <v>0.1509821790305856</v>
       </c>
       <c r="E11" t="n">
-        <v>45.41992753623194</v>
+        <v>45.41992753623193</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>-36.64384057971014</v>
       </c>
       <c r="G11" t="n">
-        <v>-36.64384057971013</v>
+        <v>0.707154309497894</v>
       </c>
       <c r="H11" t="n">
         <v>8.370652173913037</v>
       </c>
+      <c r="I11" t="n">
+        <v>0.4096613353046475</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3531,15 +3940,40 @@
         <v>0.1761604924659128</v>
       </c>
       <c r="E12" t="n">
-        <v>1035.242918024567</v>
+        <v>1035.242918024568</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>861.8928844445621</v>
       </c>
       <c r="G12" t="n">
-        <v>861.8928844445813</v>
+        <v>2.768636184734516e-30</v>
       </c>
       <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3564,12 +3998,37 @@
       <c r="F13" t="n">
         <v>0</v>
       </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>-6.725609756097933</v>
       </c>
+      <c r="I13" t="n">
+        <v>0.9874823954623538</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3594,10 +4053,33 @@
       <c r="F14" t="n">
         <v>0</v>
       </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3611,23 +4093,50 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.05212390015351587</v>
+        <v>0.05212390015351576</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2283065924442741</v>
+        <v>0.2283065924442738</v>
       </c>
       <c r="E15" t="n">
         <v>165.3170731707318</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>-45.02439024390247</v>
       </c>
       <c r="G15" t="n">
-        <v>-45.02439024390244</v>
+        <v>0.4466110323332894</v>
       </c>
       <c r="H15" t="n">
         <v>14.76829268292678</v>
       </c>
+      <c r="I15" t="n">
+        <v>0.5286356167786462</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3647,15 +4156,40 @@
         <v>0.2987461612942911</v>
       </c>
       <c r="E16" t="n">
-        <v>1120.055555555556</v>
+        <v>1120.055555555555</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>378.9444444444434</v>
       </c>
       <c r="G16" t="n">
-        <v>378.9444444444446</v>
+        <v>3.279387785137026e-05</v>
       </c>
       <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3680,12 +4214,37 @@
       <c r="F17" t="n">
         <v>0</v>
       </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>1.820598006644517</v>
       </c>
+      <c r="I17" t="n">
+        <v>0.0006587341732058186</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3708,14 +4267,41 @@
         <v>3961.48389186015</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>-3880.596677624195</v>
       </c>
       <c r="G18" t="n">
-        <v>-3880.596677624195</v>
+        <v>0.1641487704554308</v>
       </c>
       <c r="H18" t="n">
-        <v>35.05639288201944</v>
-      </c>
+        <v>35.0563928820193</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.7266658281833832</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3733,15 +4319,38 @@
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>75.460465116279</v>
+        <v>75.46046511627905</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3761,17 +4370,44 @@
         <v>0.5570382640363932</v>
       </c>
       <c r="E20" t="n">
-        <v>1248.307964601771</v>
+        <v>1248.30796460177</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>2739.642477876107</v>
       </c>
       <c r="G20" t="n">
-        <v>2739.642477876106</v>
+        <v>0.1076688253272862</v>
       </c>
       <c r="H20" t="n">
-        <v>248.3663716814161</v>
-      </c>
+        <v>248.3663716814163</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.4908409028586957</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3794,12 +4430,37 @@
         <v>1011</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>334.5000000000005</v>
       </c>
       <c r="G21" t="n">
-        <v>334.5000000000002</v>
+        <v>0.5550767070076179</v>
       </c>
       <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>